<commit_message>
fix: categories to take 2nd sheet
</commit_message>
<xml_diff>
--- a/mica/NFDI4Health.ACTIVE_P1.R-dictionary.xlsx
+++ b/mica/NFDI4Health.ACTIVE_P1.R-dictionary.xlsx
@@ -9417,7 +9417,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -9428,30 +9428,25 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>valueType</t>
+          <t>missing</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>missing</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>code</t>
         </is>
@@ -9463,25 +9458,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Participant identification number</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9493,25 +9483,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SEX</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sex</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9523,25 +9508,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B4">
-        <v>3</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AGE_BASE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Age at exposure measure [years]</t>
-        </is>
+          <t>Early Childhood Education</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>0</v>
       </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9553,25 +9533,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B5">
-        <v>4</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>EDU_LEVEL</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Highest level of education [ISCED 2011]</t>
-        </is>
+          <t>Primary Education</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9583,25 +9558,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B6">
-        <v>5</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TOT_PA_QX</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Physical activity from questionnaire data [MET-hr/day]</t>
-        </is>
+          <t>Lower Secondary Education</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9613,25 +9583,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B7">
-        <v>6</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SMOKE_ST</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Smoking status</t>
-        </is>
+          <t>Upper Secondary Education</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>3</v>
       </c>
       <c r="E7" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9643,25 +9608,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B8">
-        <v>7</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BMI</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Body Mass Index at baseline [kg/m²]</t>
-        </is>
+          <t>Post-secondary non-tertiary education</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9673,25 +9633,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B9">
-        <v>8</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ENERGY</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Energy intake [kcal/d]</t>
-        </is>
+          <t>Short-Cycle Tertiary Education</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>5</v>
       </c>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9703,25 +9658,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B10">
-        <v>9</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>POTATOES_TUB_01</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Intake of starchy roots or tubers [g/d]</t>
-        </is>
+          <t>Bachelor's or equivalent level</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>6</v>
       </c>
       <c r="E10" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9733,25 +9683,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B11">
-        <v>10</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>POTATOES_0101</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Potato intake [g/d]</t>
-        </is>
+          <t>Master's or equivalent level</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>7</v>
       </c>
       <c r="E11" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9763,25 +9708,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B12">
-        <v>11</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OTHERTUB_0102</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Other roots and tuber intake [g/d]</t>
-        </is>
+          <t>Doctoral or equivalent level</t>
+        </is>
+      </c>
+      <c r="D12">
+        <v>8</v>
       </c>
       <c r="E12" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9793,25 +9733,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B13">
-        <v>12</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EDU_LEVEL</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>VEGETABLES_02</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Vegetable intake [g/d]</t>
-        </is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D13">
+        <v>9</v>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9823,25 +9758,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B14">
-        <v>13</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SMOKE_ST</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LEAFYVEG_0201</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Leafy vegetable intake [g/d]</t>
-        </is>
+          <t>never</t>
+        </is>
+      </c>
+      <c r="D14">
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9853,25 +9783,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B15">
-        <v>14</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SMOKE_ST</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FRUITINGVEG_0202</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Fruiting vegetable intake [g/d]</t>
-        </is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D15">
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9883,25 +9808,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B16">
-        <v>15</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SMOKE_ST</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ROOTVEG_0203</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Root and tuber vegetable intake [g/d]</t>
-        </is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="D16">
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9913,25 +9833,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B17">
-        <v>16</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SMOKE_ST</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CABBAGE_0204</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Head cabbages and similar intake [g/d]</t>
-        </is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="D17">
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9943,25 +9858,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B18">
-        <v>17</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MUSHROOMS_0205</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Mushroom intake [g/d]</t>
-        </is>
+          <t>FPQ (Food propensity questionnair without portion sizes)</t>
+        </is>
+      </c>
+      <c r="D18">
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -9973,25 +9883,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B19">
-        <v>18</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRAINPODVEG_0206</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Intake of legumes with pod [g/d]</t>
-        </is>
+          <t>FFQ (Food frequency questionnaire)</t>
+        </is>
+      </c>
+      <c r="D19">
+        <v>1</v>
       </c>
       <c r="E19" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -10003,25 +9908,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B20">
-        <v>19</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ONION_GARLIC_0207</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Bulb vegetables (onions, garlic) intake [g/d]</t>
-        </is>
+          <t>24HDR (24-h dietary recall)</t>
+        </is>
+      </c>
+      <c r="D20">
+        <v>2</v>
       </c>
       <c r="E20" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -10033,25 +9933,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B21">
-        <v>20</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>STALKVEG_0208</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Intake of stems/stalks eaten as vegetables [g/d]</t>
-        </is>
+          <t>3_d_FR_w (3-day weighing food record)</t>
+        </is>
+      </c>
+      <c r="D21">
+        <v>3</v>
       </c>
       <c r="E21" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -10063,25 +9958,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B22">
-        <v>21</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MIXEDVEG_0209</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Intake of mixed vegetable salad or mixed green salad [g/d]</t>
-        </is>
+          <t>7_d_FR (7-day  food record; described portion sizes)</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>4</v>
       </c>
       <c r="E22" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -10093,25 +9983,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B23">
-        <v>22</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LEGUMES_TOT_03</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Total legumes intake [g/d]</t>
-        </is>
+          <t>7_d_FR_w (7-day weighing food record)</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>5</v>
       </c>
       <c r="E23" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -10123,3175 +10008,20 @@
           <t>ACTIVE_P1</t>
         </is>
       </c>
-      <c r="B24">
-        <v>23</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DIETARY_ASSESS_INSTR</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LEGUMES_0301</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Intake fresh seeds (without pod) from legumes (beans, peas etc.) [g/d]</t>
-        </is>
+          <t>24HFL_FFQ (24-h short food list combined with FFQ)</t>
+        </is>
+      </c>
+      <c r="D24">
+        <v>6</v>
       </c>
       <c r="E24" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B25">
-        <v>24</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>FRUITS_TOT_04</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Total fruit intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B26">
-        <v>25</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>FRUITS_0401</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Intake of fresh fruits [g/d]</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B27">
-        <v>26</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>NUTS_SEEDS_0402</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Intake of tree nuts and seeds [g/d]</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B28">
-        <v>27</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>MIXEDFRUITS_0403</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Intake of candied fruit/mixed fruit, canned, jarred mixed fruit and miscellaneous fruits [g/d]</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B29">
-        <v>28</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>OLIVES_0404</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Intake of olives [g/d]</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B30">
-        <v>29</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>DAIRY_05</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Intake of milk and dairy products and milk and milk products (dairy) [g/d]</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B31">
-        <v>30</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>MILK_0501</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Intake of (whole) cow and cattle milk [g/d]</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B32">
-        <v>31</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>MILKBEV_0502</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Intake of buttermilk, traditional buttermilk, flavoured milk, flavoured whey and milk-based drinks (as part-nature) [g/d]</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B33">
-        <v>32</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>YOGURT_0503</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Intake of fermented milk products [g/d]</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B34">
-        <v>33</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>CURD_0504</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Intake of cheese curd, quark and cottage [g/d]</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B35">
-        <v>34</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>CHEESE_0505</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Intake of cheese [g/d]</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B36">
-        <v>35</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>DAIRYDESSERT_0506</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Intake of dairy dessert and similar starchy pudding [g/d]</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B37">
-        <v>36</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>CREAM_PROD_0507</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Intake of cream and cream products [g/d]</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B38">
-        <v>37</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>DAIRYCREAM_050701</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Cream intake (as part-nature) [g/d]</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B39">
-        <v>38</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>NONDAIRYCREAM_050702</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Intake of imitation cream, non-dairy coffee creamers and dairy imitates other than milk [g/d]</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B40">
-        <v>39</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MILK_FOR_COFFEE_0508</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Intake of condensed milk (sometimes with added sugars) and milk and dairy powders and concentrates [g/d]</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B41">
-        <v>40</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>CEREAL_PROD_06</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Intake of cereals and cereal primary derivatives, cereal grains (and cereal-like grains) [g/d]</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B42">
-        <v>41</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>FLOUR_FLAKES_0601</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Intake of flours and other milled products and starches [g/d]</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B43">
-        <v>42</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>PASTA_RICE_0602</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Intake of pastas and rice [g/d]</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B44">
-        <v>43</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>BREAD_PROD_0603</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Intake of bread and bread products [g/d]</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B45">
-        <v>44</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>BREAD_060301</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Intake of bread [g/d]</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B46">
-        <v>45</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>CRISPBREAD_060302</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Intake of crisp bread and rusk [g/d]</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B47">
-        <v>46</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>BREAKF_CEREALS_0604</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Intake of breakfast cereals [g/d]</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B48">
-        <v>47</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>SALT_BISCUIT_0605</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Intake of crackers and breadsticks [g/d]</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B49">
-        <v>48</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>DOUGH_PASTRY_0606</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Intake of fine bakery products [g/d]</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B50">
-        <v>49</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>MEAT_PROD_07</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Intake of meat and meat products [g/d]</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B51">
-        <v>50</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>RED_MEAT_0701</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Intake of red meat (mammals meat) [g/d]</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B52">
-        <v>51</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>BEEF_070101</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Intake of cow, ox or bull fresh meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B53">
-        <v>52</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>VEAL_070102</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Intake of calf fresh meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B54">
-        <v>53</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>PORK_070103</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Intake of pig fresh meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B55">
-        <v>54</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>MUTTON_LAMB_070104</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Intake of lamb and sheep meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B56">
-        <v>55</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>HORSE_070105</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Intake of horse meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B57">
-        <v>56</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>GOAT_070106</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Intake of goat meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B58">
-        <v>57</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>POULTRY_0702</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Intake of poultry meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B59">
-        <v>58</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>OTHERPOULTRY_070200</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Intake of other poultry meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B60">
-        <v>59</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>CHICKEN_070201</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Intake of chicken meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B61">
-        <v>60</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>TURKEY_070202</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Intake of turkey meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B62">
-        <v>61</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>DUCK_070203</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Intake of duck meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B63">
-        <v>62</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>GOOSE_070204</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Intake of goose meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B64">
-        <v>63</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>RABBIT_070205</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Intake of rabbit meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B65">
-        <v>64</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>GAME_0703</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Intake of game [g/d]</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B66">
-        <v>65</v>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>PROCMEAT_0704</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Intake of processed or preserved meat [g/d]</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B67">
-        <v>66</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>OFFALS_0705</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Intake of animal offal and other slaughtering [g/d]</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B68">
-        <v>67</v>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>FISH_SHELLFISH_08</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Intake of fish and seafood and products thereof [g/d]</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B69">
-        <v>68</v>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>FISH_0801</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Intake of fish (meat) [g/d]</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B70">
-        <v>69</v>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>CRUSTACEANS_0802</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Intake of seafood and products thereof [g/d]</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B71">
-        <v>70</v>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>FISH_PROD_0803</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Intake of processed fish [g/d]</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B72">
-        <v>71</v>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>EGG_PROD_09</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Intake of eggs and egg products [g/d]</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B73">
-        <v>72</v>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>EGGS_0901</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Intake of eggs [g/d]</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B74">
-        <v>73</v>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>FAT_10</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Intake of animal and vegetable fats and oils [g/d]</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B75">
-        <v>74</v>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>VEGOILS_1001</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Intake of vegetable fats and oils [g/d]</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B76">
-        <v>75</v>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>BUTTER_1002</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Intake of butter [g/d]</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B77">
-        <v>76</v>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>MARGARINE_1003</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Intake of margarines and similar [g/d]</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B78">
-        <v>77</v>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>FRYFAT_1004</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Intake of blended frying oil/fats [g/d]</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B79">
-        <v>78</v>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>MARINEOILS_1005</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Intake of fats and oils from marine sources [g/d]</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B80">
-        <v>79</v>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>OTHER_ANIMALFAT_1006</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Intake of animal fats (processed fat from animal tissue) [g/d]</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B81">
-        <v>80</v>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>SUGAR_CONFECT_11</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Intake of sugar and similar, confectionery and water-based sweet desserts [g/d]</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B82">
-        <v>81</v>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>HONEY_JAM_1101</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Intake of sugars, syrups, honey and table-top sweeteners [g/d]</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B83">
-        <v>82</v>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>CHOCOLATE_1102</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Intake of chocolate, chocolate products and chocolate coated confectionary [g/d]</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B84">
-        <v>83</v>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>NONCHOC_SWEETS_1103</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Intake of sweet bars and other formed sweet masses, candies (soft and hard) and other confectionery including breath refreshening microsweets [g/d]</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B85">
-        <v>84</v>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>SYRUP_1104</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Intake of corn syrup and sugar beet syrup [g/d]</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B86">
-        <v>85</v>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>ICECREAM_1105</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Intake of spoonable desserts and ice creams [g/d]</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B87">
-        <v>86</v>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>ICECREAM_MILK_110501</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Intake of milk-based ice cream [g/d]</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B88">
-        <v>87</v>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>SORBET_110502</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Sorbet intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B89">
-        <v>88</v>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>WATER_ICE_110503</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Intake of water-based ice creams [g/d]</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B90">
-        <v>89</v>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>CAKES_12</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Intake of cakes and fine bakery products [g/d]</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B91">
-        <v>90</v>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>VARPASTRY_1201</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>Intake of various pastry [g/d]</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B92">
-        <v>91</v>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>DRYCAKE_1202</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>Intake of sponge biscuits and plain cakes [g/d]</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B93">
-        <v>92</v>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>NONALC_BEV_13</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Intake of non-alcoholic beverages [g/d]</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B94">
-        <v>93</v>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>FRUITVEG_JUICE_1301</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Intake of fruit and vegetable juices [g/d]</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B95">
-        <v>94</v>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>SOFTDRINKS_1302</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Intake of soft drinks [g/d]</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B96">
-        <v>95</v>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>HOTDRINKS_1303</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>Intake of hot drinks and similar (coffee, cocoa, tea and herbal infusions) [g/d]</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B97">
-        <v>96</v>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>COFFEE_130301</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Coffee intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B98">
-        <v>97</v>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>TEA_130302</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Tea intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B99">
-        <v>98</v>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>HERBALTEA_130303</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Intake of herbal and other non-tea infusions [g/d]</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B100">
-        <v>99</v>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>COFFEE_IMITATE_130304</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Intake of chicory coffee infusion and coffee imitate beverages [g/d]</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B101">
-        <v>100</v>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>WATER_1304</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Intake of water and water-based beverages [g/d]</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B102">
-        <v>101</v>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>ALC_BEV_14</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Alcoholic beverage intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B103">
-        <v>102</v>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>WINE_1401</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>Intake of wine and wine-like drinks [g/d]</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B104">
-        <v>103</v>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>FORTWINE_1402</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Intake of fortified/liqueur wine [g/d]</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B105">
-        <v>104</v>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>BEER_1403</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Intake of beer and beer-like beverage [g/d]</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B106">
-        <v>105</v>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>SPIRITS_1404</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Intake of unsweetened spirits [g/d]</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B107">
-        <v>106</v>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>HERBLIQUEUR_1405</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>Intake of herb liqueur [g/d]</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B108">
-        <v>107</v>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>LIQUEURS_1406</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Intake of liqueurs [g/d]</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B109">
-        <v>108</v>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>COCKTAILS_1407</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Intake of mixed alcoholic drinks [g/d]</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B110">
-        <v>109</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>CONDIMENT_SAUCES_15</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Intake of seasoning, sauces and condiments [g/d]</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B111">
-        <v>110</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>SAUCES_1501</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Intake of savoury sauces [g/d]</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B112">
-        <v>111</v>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>TOMATOSAUCE_150101</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Intake of tomato-containing cooked sauces [g/d]</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B113">
-        <v>112</v>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>DRESSINGS_150102</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Dressing intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B114">
-        <v>113</v>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>MAYONNAISE_150103</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Intake of mayonnaise [g/d]</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B115">
-        <v>114</v>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>DESSERTSAUCE_150104</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Intakes of dessert sauces/toppings [g/d]</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B116">
-        <v>115</v>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>YEAST_1502</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Intake of yeast cultures [g/d]</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B117">
-        <v>116</v>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>HERBS_SPICES_1503</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Intakes of berbs, spices and similar [g/d]</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B118">
-        <v>117</v>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>CONDIMENTS_1504</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>Condiments intake [g/d]</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B119">
-        <v>118</v>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>SOUP_BOUILLON_16</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Intake of soups and broths [g/d]</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B120">
-        <v>119</v>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>SOUP_1601</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>Intake of soups [g/d]</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B121">
-        <v>120</v>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>BOUILLON_1602</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>Intake of mixed vegetables soup, clear meat soup [g/d]</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B122">
-        <v>121</v>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>MISCELLANEOUS_17</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Intake of miscellaneous [g/d]</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B123">
-        <v>122</v>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>VEG_DISHES_1700</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>Intake of vegetarian products and dishes [g/d]</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B124">
-        <v>123</v>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>SOY_PROD_1701</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>Intake of soy products [g/d]</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B125">
-        <v>124</v>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>DIET_PROD_1702</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>Intake of food for weight reduction [g/d]</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B126">
-        <v>125</v>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>ART_SWEETENER_170201</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Intake of artificial sweeteners (e.g., aspartam, saccharine) [g/d]</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B127">
-        <v>126</v>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>SNACKS_1703</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Intake of snacks other than chips and similar [g/d]</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B128">
-        <v>127</v>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>AMPHIBIANS_1704</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Intake of amphibians, reptiles, snails, insects [g/d]</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>decimal</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>ACTIVE_P1</t>
-        </is>
-      </c>
-      <c r="B129">
-        <v>128</v>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>DIETARY_ASSESS_INSTR</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Dietary Assessment Instrument</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>